<commit_message>
MacLarnon folder renamed to fit system, so files were moved. Also Project Kaskan updates
</commit_message>
<xml_diff>
--- a/____Unpublished__ProjectKaskan/unique_area_names.xlsx
+++ b/____Unpublished__ProjectKaskan/unique_area_names.xlsx
@@ -989,9 +989,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EB21CDC-66F1-4E15-A200-A282BDB4F01B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BE36B1E-8C42-42A6-9A37-1AB7759BAF82}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{521D4E9D-23BF-45F2-AE23-B3117182DB3A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46F644BC-5DD4-480E-A880-DBE6D0018349}"/>
 </file>
</xml_diff>